<commit_message>
auto refresh, penalty & suprise bonus calculation
</commit_message>
<xml_diff>
--- a/UAT Testing Tracker.xlsx
+++ b/UAT Testing Tracker.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\auction-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD6F865-5A1B-4BD8-8AB9-2E00C76A2FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF8554E-5C0A-45C2-B86E-A8A8A071F41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{04BEFEA4-68C6-4061-9385-558C75477688}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{04BEFEA4-68C6-4061-9385-558C75477688}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="tester_sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="clean_sheet" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="57">
   <si>
     <t>1. Fielding dismissals nhi dikh rha</t>
   </si>
@@ -126,26 +127,111 @@
     <t>need to check with admin once more</t>
   </si>
   <si>
-    <t>will reflect after sync data</t>
-  </si>
-  <si>
     <t>reflecting</t>
   </si>
   <si>
-    <t>will work post deployment</t>
+    <t>need to restart auction</t>
+  </si>
+  <si>
+    <t>Missing fielding_dismissals columns</t>
+  </si>
+  <si>
+    <t>Integer should be shown as integer not float</t>
+  </si>
+  <si>
+    <t>Innings column not reflecting</t>
+  </si>
+  <si>
+    <t>photo name and player names are different for certain players, not rendering profile pic properly</t>
+  </si>
+  <si>
+    <t>database transaction like saving surprise player or prediction tax player are taking too much time to reflect</t>
+  </si>
+  <si>
+    <t>Not Done</t>
+  </si>
+  <si>
+    <t>multiple people accessing admin and doing same database transaction</t>
+  </si>
+  <si>
+    <t>Manual refresh is needed after every transaction not good UI/UX experience for admin and captains</t>
+  </si>
+  <si>
+    <t>9. During spin wheel it takes some time to present the spin effect or putting the player on block.</t>
+  </si>
+  <si>
+    <t>Need a popup message for admin to see after surprise player is sold and prediction tax player is sold, backend tax deduction and bonus calculation is happening but not notification</t>
+  </si>
+  <si>
+    <t>Need a separate penalty  tax player details like surprise player list</t>
+  </si>
+  <si>
+    <t>after each player sold instead of wheel the page refresh and goes to manage team tab for admi</t>
+  </si>
+  <si>
+    <t>marquee nomination can be seen by everyone</t>
+  </si>
+  <si>
+    <t>no code changes required</t>
+  </si>
+  <si>
+    <t>require code changes</t>
+  </si>
+  <si>
+    <t>code changes done need a verification</t>
+  </si>
+  <si>
+    <t>Floor Logic Anomaly on Surprise Player Bonuses</t>
+  </si>
+  <si>
+    <t>Floor Logic Anomaly on Prediction Tax Player</t>
+  </si>
+  <si>
+    <t>bsence of Administrative Transaction Reversal Framework (Undo Last Sale)</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Navbar issue, due to dark theme of the app once the navbar is collapsed the arrow is not visible so an admin or captain can't use the navbar to refresh data or logout properly especially if they are using phone</t>
+  </si>
+  <si>
+    <t>Certain design like player card not rendering well espcially on phone view espcially after addition of fielding &amp; inning data</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF569CD6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -174,9 +260,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,243 +583,606 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43A76C7C-7072-407A-B7A5-86F6224BB5E6}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="129.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="50.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="1"/>
-      <c r="C21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D21" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C21" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B25" s="1"/>
-      <c r="C25" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D25" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30608C33-0D76-4BC9-BC62-BB6EE057613C}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>